<commit_message>
Updated all namespces to be Einsatzplanung.something. Updeated GeneratorService. Added data types for plan generation.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Aubilder.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Aubilder.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756D4D80-A4A8-4AAB-8143-F4DC245F1BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816CEA83-C6E5-4084-95D2-11FF9909EB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>Programmierung</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Sb</t>
   </si>
   <si>
-    <t>IT-Systeme &amp; Administration</t>
-  </si>
-  <si>
     <t>Sch</t>
   </si>
   <si>
@@ -98,28 +95,19 @@
     <t>Wochenstunden</t>
   </si>
   <si>
-    <t>Netzwerke &amp; Dienste</t>
-  </si>
-  <si>
     <t>Pruefungsvorbereitung</t>
   </si>
   <si>
     <t>Grundlagen</t>
   </si>
   <si>
-    <t>IT-Systeme &amp; Grundlagen</t>
-  </si>
-  <si>
-    <t>Programmierung &amp; Projektmanagement</t>
-  </si>
-  <si>
     <t>Projektmanagement</t>
   </si>
   <si>
-    <t>Netzwerke &amp; IT-Sicherheit</t>
-  </si>
-  <si>
     <t>IT-Sicherheit</t>
+  </si>
+  <si>
+    <t>Dienste</t>
   </si>
 </sst>
 </file>
@@ -491,11 +479,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA7A25F-1A13-43E6-8B5A-038B5C3A6F73}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="65.42578125" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -507,10 +495,10 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -521,7 +509,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>40</v>
@@ -533,104 +521,89 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>20</v>
+      <c r="D7">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9">
         <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11">
         <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C11" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Ausbilder.xlsx and Lehrjahre.slsx for easier testing.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Aubilder.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Aubilder.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362DA868-56B2-4E20-A7ED-2025B4B8AD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579E79D1-5A78-49AD-9100-7B9EA1260139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="555" windowWidth="13170" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>Programmierung</t>
   </si>
@@ -479,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA7A25F-1A13-43E6-8B5A-038B5C3A6F73}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" customWidth="1"/>
@@ -528,7 +528,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4">
         <v>40</v>
@@ -536,42 +536,33 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
       <c r="C7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D9">
         <v>40</v>
@@ -579,30 +570,59 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12">
         <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C12" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>